<commit_message>
finish the group comparisons: trait links, module preservation and cluster phenotype as walkthroughs
</commit_message>
<xml_diff>
--- a/03_Group_comparisons/HRvLR/07_Module_Preservation/c_data/module_preservation.xlsx
+++ b/03_Group_comparisons/HRvLR/07_Module_Preservation/c_data/module_preservation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11941" uniqueCount="2157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11950" uniqueCount="2163">
   <si>
     <t>sheet</t>
   </si>
@@ -6247,6 +6247,12 @@
     <t>1.0.14</t>
   </si>
   <si>
+    <t>jsonlite</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
+  </si>
+  <si>
     <t>knitr</t>
   </si>
   <si>
@@ -6463,6 +6469,12 @@
     <t>0.5.0</t>
   </si>
   <si>
+    <t>utf8</t>
+  </si>
+  <si>
+    <t>1.2.6</t>
+  </si>
+  <si>
     <t>vctrs</t>
   </si>
   <si>
@@ -6491,6 +6503,12 @@
   </si>
   <si>
     <t>0.57</t>
+  </si>
+  <si>
+    <t>yaml</t>
+  </si>
+  <si>
+    <t>2.3.12</t>
   </si>
 </sst>
 </file>
@@ -50103,7 +50121,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -50639,7 +50657,7 @@
         <v>2081</v>
       </c>
       <c r="B49" t="s">
-        <v>2029</v>
+        <v>2082</v>
       </c>
       <c r="C49" t="s">
         <v>1988</v>
@@ -50647,10 +50665,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>2082</v>
+        <v>2083</v>
       </c>
       <c r="B50" t="s">
-        <v>2083</v>
+        <v>2029</v>
       </c>
       <c r="C50" t="s">
         <v>1988</v>
@@ -50741,7 +50759,7 @@
         <v>2099</v>
       </c>
       <c r="C58" t="s">
-        <v>1993</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="59" spans="1:3">
@@ -50752,7 +50770,7 @@
         <v>2101</v>
       </c>
       <c r="C59" t="s">
-        <v>1988</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="60" spans="1:3">
@@ -50826,10 +50844,10 @@
         <v>2114</v>
       </c>
       <c r="B66" t="s">
-        <v>2033</v>
+        <v>2115</v>
       </c>
       <c r="C66" t="s">
-        <v>2115</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -50837,10 +50855,10 @@
         <v>2116</v>
       </c>
       <c r="B67" t="s">
+        <v>2033</v>
+      </c>
+      <c r="C67" t="s">
         <v>2117</v>
-      </c>
-      <c r="C67" t="s">
-        <v>1988</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -50884,7 +50902,7 @@
         <v>2125</v>
       </c>
       <c r="C71" t="s">
-        <v>1993</v>
+        <v>1988</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -50895,7 +50913,7 @@
         <v>2127</v>
       </c>
       <c r="C72" t="s">
-        <v>1988</v>
+        <v>1993</v>
       </c>
     </row>
     <row r="73" spans="1:3">
@@ -50991,7 +51009,7 @@
         <v>2144</v>
       </c>
       <c r="B81" t="s">
-        <v>2025</v>
+        <v>2145</v>
       </c>
       <c r="C81" t="s">
         <v>1988</v>
@@ -50999,10 +51017,10 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>2145</v>
+        <v>2146</v>
       </c>
       <c r="B82" t="s">
-        <v>2146</v>
+        <v>2025</v>
       </c>
       <c r="C82" t="s">
         <v>1988</v>
@@ -51060,6 +51078,39 @@
         <v>2156</v>
       </c>
       <c r="C87" t="s">
+        <v>1988</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3">
+      <c r="A88" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B88" t="s">
+        <v>2158</v>
+      </c>
+      <c r="C88" t="s">
+        <v>1988</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3">
+      <c r="A89" t="s">
+        <v>2159</v>
+      </c>
+      <c r="B89" t="s">
+        <v>2160</v>
+      </c>
+      <c r="C89" t="s">
+        <v>1988</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3">
+      <c r="A90" t="s">
+        <v>2161</v>
+      </c>
+      <c r="B90" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C90" t="s">
         <v>1988</v>
       </c>
     </row>

</xml_diff>